<commit_message>
Refresh final reviewed subsystem workbooks
</commit_message>
<xml_diff>
--- a/samples/ss_prbc_ingest.xlsx
+++ b/samples/ss_prbc_ingest.xlsx
@@ -845,7 +845,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2,4</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -916,7 +916,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>

</xml_diff>